<commit_message>
Actualización automática 2026-01-21 08:30:10
</commit_message>
<xml_diff>
--- a/data/MEZA PEÑA CARLOS ROBERTO.xlsx
+++ b/data/MEZA PEÑA CARLOS ROBERTO.xlsx
@@ -1405,7 +1405,7 @@
         <v>0</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>172.99</v>
+        <v>630.91</v>
       </c>
       <c r="E16" s="2" t="n">
         <v>0</v>
@@ -1429,7 +1429,7 @@
         <v>0</v>
       </c>
       <c r="L16" s="2" t="n">
-        <v>443.44</v>
+        <v>591.25</v>
       </c>
       <c r="M16" s="2" t="n">
         <v>0</v>
@@ -2351,7 +2351,7 @@
         <v>96.37</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>616.4299999999999</v>
+        <v>1222.16</v>
       </c>
       <c r="G16" s="2" t="n">
         <v>0</v>
@@ -2530,7 +2530,7 @@
         <v>96.37</v>
       </c>
       <c r="F23" s="4" t="n">
-        <v>11079.71</v>
+        <v>11685.44</v>
       </c>
       <c r="G23" s="4" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Actualización automática 2026-01-27 13:30:13
</commit_message>
<xml_diff>
--- a/data/MEZA PEÑA CARLOS ROBERTO.xlsx
+++ b/data/MEZA PEÑA CARLOS ROBERTO.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R27"/>
+  <dimension ref="A1:R32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1038,7 +1038,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>FERRETERIA UNIDA ZAMBRANO FERRUZAM CIA. LTDA.</t>
+          <t>DELGADO COPPIANO JORGE RODOLFO</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
@@ -1098,7 +1098,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>FREILE FERRIN FRECIA NOEMI LOURDE</t>
+          <t>DELGADO LOOR JORGE ARTURO</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>GONZALEZ CARDENAS ERNESTO PAOLO</t>
+          <t>DISALME CIA. LTDA.</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
@@ -1218,7 +1218,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>GRANIMUNDO S.A.</t>
+          <t>FERRETERIA UNIDA ZAMBRANO FERRUZAM CIA. LTDA.</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
@@ -1228,7 +1228,7 @@
         <v>0</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>166.61</v>
+        <v>0</v>
       </c>
       <c r="F13" s="2" t="n">
         <v>0</v>
@@ -1278,7 +1278,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>LINO TUMBACO VICENTE JAVIER</t>
+          <t>FREILE FERRIN FRECIA NOEMI LOURDE</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
@@ -1312,7 +1312,7 @@
         <v>0</v>
       </c>
       <c r="M14" s="2" t="n">
-        <v>1496.72</v>
+        <v>0</v>
       </c>
       <c r="N14" s="2" t="n">
         <v>0</v>
@@ -1338,7 +1338,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>MANABITA DE REPUESTOS MANARECO C LTDA</t>
+          <t>GONZALEZ CARDENAS ERNESTO PAOLO</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
@@ -1398,7 +1398,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>MATERIALES PARA DECORACION DECORCASA CIA. LTDA.</t>
+          <t>GRANIMUNDO S.A.</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
@@ -1408,7 +1408,7 @@
         <v>0</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>0</v>
+        <v>166.61</v>
       </c>
       <c r="F16" s="2" t="n">
         <v>0</v>
@@ -1432,7 +1432,7 @@
         <v>0</v>
       </c>
       <c r="M16" s="2" t="n">
-        <v>3124.48</v>
+        <v>0</v>
       </c>
       <c r="N16" s="2" t="n">
         <v>0</v>
@@ -1458,17 +1458,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>MOREIRA MOREIRA PATRICIO IGNACIO</t>
+          <t>LINO TUMBACO VICENTE JAVIER</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>1166.4</v>
+        <v>0</v>
       </c>
       <c r="D17" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>867.5599999999999</v>
+        <v>0</v>
       </c>
       <c r="F17" s="2" t="n">
         <v>0</v>
@@ -1489,10 +1489,10 @@
         <v>0</v>
       </c>
       <c r="L17" s="2" t="n">
-        <v>2345.61</v>
+        <v>0</v>
       </c>
       <c r="M17" s="2" t="n">
-        <v>1496.14</v>
+        <v>1496.72</v>
       </c>
       <c r="N17" s="2" t="n">
         <v>0</v>
@@ -1518,14 +1518,14 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>PAREDES ORTIZ MARIA INES</t>
+          <t>MANABITA DE REPUESTOS MANARECO C LTDA</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>2719.84</v>
+        <v>0</v>
       </c>
       <c r="E18" s="2" t="n">
         <v>0</v>
@@ -1578,14 +1578,14 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>RENOVA&amp;DISEÑA S.A.</t>
+          <t>MATERIALES PARA DECORACION DECORCASA CIA. LTDA.</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>630.91</v>
+        <v>0</v>
       </c>
       <c r="E19" s="2" t="n">
         <v>0</v>
@@ -1609,10 +1609,10 @@
         <v>0</v>
       </c>
       <c r="L19" s="2" t="n">
-        <v>591.25</v>
+        <v>0</v>
       </c>
       <c r="M19" s="2" t="n">
-        <v>0</v>
+        <v>3124.48</v>
       </c>
       <c r="N19" s="2" t="n">
         <v>0</v>
@@ -1638,17 +1638,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>REYES AGUILERA JESSICA ELIZABETH</t>
+          <t>MOREIRA MOREIRA PATRICIO IGNACIO</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>0</v>
+        <v>1166.4</v>
       </c>
       <c r="D20" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>0</v>
+        <v>867.5599999999999</v>
       </c>
       <c r="F20" s="2" t="n">
         <v>0</v>
@@ -1669,10 +1669,10 @@
         <v>0</v>
       </c>
       <c r="L20" s="2" t="n">
-        <v>0</v>
+        <v>2345.61</v>
       </c>
       <c r="M20" s="2" t="n">
-        <v>0</v>
+        <v>1496.14</v>
       </c>
       <c r="N20" s="2" t="n">
         <v>0</v>
@@ -1698,14 +1698,14 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>ROCA REYNA PAUL DAVID</t>
+          <t>PAREDES ORTIZ MARIA INES</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>0</v>
+        <v>2719.84</v>
       </c>
       <c r="E21" s="2" t="n">
         <v>0</v>
@@ -1758,14 +1758,14 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>SUMBA GARCIA MARCOS ANTONIO</t>
+          <t>RENOVA&amp;DISEÑA S.A.</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>0</v>
+        <v>630.91</v>
       </c>
       <c r="E22" s="2" t="n">
         <v>0</v>
@@ -1789,7 +1789,7 @@
         <v>0</v>
       </c>
       <c r="L22" s="2" t="n">
-        <v>0</v>
+        <v>591.25</v>
       </c>
       <c r="M22" s="2" t="n">
         <v>0</v>
@@ -1818,7 +1818,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>TUTIVEN PAREDES MARCIA PIEDAD</t>
+          <t>REYES AGUILERA JESSICA ELIZABETH</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
@@ -1878,7 +1878,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>VACA CANCHINGRE FATIMA YAQUELINE</t>
+          <t>ROCA REYNA PAUL DAVID</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
@@ -1938,7 +1938,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>ZAMBRANO FERNANDEZ JOSE LUIS</t>
+          <t>SOLORZANO BRAVO TERESA CONCEPCION</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
@@ -1998,137 +1998,437 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
+          <t>SUMBA GARCIA MARCOS ANTONIO</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R26" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>MEZA PEÑA CARLOS ROBERTO</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>TUTIVEN PAREDES MARCIA PIEDAD</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R27" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>MEZA PEÑA CARLOS ROBERTO</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>VACA CANCHINGRE FATIMA YAQUELINE</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R28" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>MEZA PEÑA CARLOS ROBERTO</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>VERA ARCE MARIA ISABEL</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R29" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>MEZA PEÑA CARLOS ROBERTO</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>ZAMBRANO FERNANDEZ JOSE LUIS</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R30" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>MEZA PEÑA CARLOS ROBERTO</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
           <t>ZAMBRANO REYNA JOSE ALEJANDRO</t>
         </is>
       </c>
-      <c r="C26" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D26" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E26" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F26" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G26" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H26" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I26" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J26" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K26" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L26" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M26" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N26" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O26" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P26" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q26" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R26" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="C27" s="3" t="inlineStr">
-        <is>
-          <t>1 de 25</t>
-        </is>
-      </c>
-      <c r="D27" s="3" t="inlineStr">
-        <is>
-          <t>2 de 25</t>
-        </is>
-      </c>
-      <c r="E27" s="3" t="inlineStr">
-        <is>
-          <t>2 de 25</t>
-        </is>
-      </c>
-      <c r="F27" s="3" t="inlineStr">
-        <is>
-          <t>0 de 25</t>
-        </is>
-      </c>
-      <c r="G27" s="3" t="inlineStr">
-        <is>
-          <t>0 de 25</t>
-        </is>
-      </c>
-      <c r="H27" s="3" t="inlineStr">
-        <is>
-          <t>1 de 25</t>
-        </is>
-      </c>
-      <c r="I27" s="3" t="inlineStr">
-        <is>
-          <t>1 de 25</t>
-        </is>
-      </c>
-      <c r="J27" s="3" t="inlineStr">
-        <is>
-          <t>0 de 25</t>
-        </is>
-      </c>
-      <c r="K27" s="3" t="inlineStr">
-        <is>
-          <t>0 de 25</t>
-        </is>
-      </c>
-      <c r="L27" s="3" t="inlineStr">
-        <is>
-          <t>2 de 25</t>
-        </is>
-      </c>
-      <c r="M27" s="3" t="inlineStr">
-        <is>
-          <t>3 de 25</t>
-        </is>
-      </c>
-      <c r="N27" s="3" t="inlineStr">
-        <is>
-          <t>0 de 25</t>
-        </is>
-      </c>
-      <c r="O27" s="3" t="inlineStr">
-        <is>
-          <t>0 de 25</t>
-        </is>
-      </c>
-      <c r="P27" s="3" t="inlineStr">
-        <is>
-          <t>0 de 25</t>
-        </is>
-      </c>
-      <c r="Q27" s="3" t="inlineStr">
-        <is>
-          <t>0 de 25</t>
-        </is>
-      </c>
-      <c r="R27" s="3" t="inlineStr">
-        <is>
-          <t>0 de 25</t>
+      <c r="C31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R31" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>1 de 30</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>2 de 30</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>2 de 30</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>0 de 30</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="inlineStr">
+        <is>
+          <t>0 de 30</t>
+        </is>
+      </c>
+      <c r="H32" s="3" t="inlineStr">
+        <is>
+          <t>1 de 30</t>
+        </is>
+      </c>
+      <c r="I32" s="3" t="inlineStr">
+        <is>
+          <t>1 de 30</t>
+        </is>
+      </c>
+      <c r="J32" s="3" t="inlineStr">
+        <is>
+          <t>0 de 30</t>
+        </is>
+      </c>
+      <c r="K32" s="3" t="inlineStr">
+        <is>
+          <t>0 de 30</t>
+        </is>
+      </c>
+      <c r="L32" s="3" t="inlineStr">
+        <is>
+          <t>2 de 30</t>
+        </is>
+      </c>
+      <c r="M32" s="3" t="inlineStr">
+        <is>
+          <t>3 de 30</t>
+        </is>
+      </c>
+      <c r="N32" s="3" t="inlineStr">
+        <is>
+          <t>0 de 30</t>
+        </is>
+      </c>
+      <c r="O32" s="3" t="inlineStr">
+        <is>
+          <t>0 de 30</t>
+        </is>
+      </c>
+      <c r="P32" s="3" t="inlineStr">
+        <is>
+          <t>0 de 30</t>
+        </is>
+      </c>
+      <c r="Q32" s="3" t="inlineStr">
+        <is>
+          <t>0 de 30</t>
+        </is>
+      </c>
+      <c r="R32" s="3" t="inlineStr">
+        <is>
+          <t>0 de 30</t>
         </is>
       </c>
     </row>
@@ -2143,7 +2443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2416,7 +2716,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>FERRETERIA UNIDA ZAMBRANO FERRUZAM CIA. LTDA.</t>
+          <t>DELGADO COPPIANO JORGE RODOLFO</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
@@ -2443,7 +2743,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>FREILE FERRIN FRECIA NOEMI LOURDE</t>
+          <t>DELGADO LOOR JORGE ARTURO</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
@@ -2470,7 +2770,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>GONZALEZ CARDENAS ERNESTO PAOLO</t>
+          <t>DISALME CIA. LTDA.</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
@@ -2497,11 +2797,11 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>GRANIMUNDO S.A.</t>
+          <t>FERRETERIA UNIDA ZAMBRANO FERRUZAM CIA. LTDA.</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>1382.33</v>
+        <v>0</v>
       </c>
       <c r="D13" s="2" t="n">
         <v>0</v>
@@ -2510,7 +2810,7 @@
         <v>0</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>166.61</v>
+        <v>0</v>
       </c>
       <c r="G13" s="2" t="n">
         <v>0</v>
@@ -2524,7 +2824,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>LINO TUMBACO VICENTE JAVIER</t>
+          <t>FREILE FERRIN FRECIA NOEMI LOURDE</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
@@ -2537,7 +2837,7 @@
         <v>0</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>1496.72</v>
+        <v>0</v>
       </c>
       <c r="G14" s="2" t="n">
         <v>0</v>
@@ -2551,7 +2851,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>MANABITA DE REPUESTOS MANARECO C LTDA</t>
+          <t>GONZALEZ CARDENAS ERNESTO PAOLO</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
@@ -2578,20 +2878,20 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>MATERIALES PARA DECORACION DECORCASA CIA. LTDA.</t>
+          <t>GRANIMUNDO S.A.</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>0</v>
+        <v>1382.33</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>835.22</v>
+        <v>0</v>
       </c>
       <c r="E16" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>3124.48</v>
+        <v>166.61</v>
       </c>
       <c r="G16" s="2" t="n">
         <v>0</v>
@@ -2605,11 +2905,11 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>MOREIRA MOREIRA PATRICIO IGNACIO</t>
+          <t>LINO TUMBACO VICENTE JAVIER</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>89.76000000000001</v>
+        <v>0</v>
       </c>
       <c r="D17" s="2" t="n">
         <v>0</v>
@@ -2618,7 +2918,7 @@
         <v>0</v>
       </c>
       <c r="F17" s="2" t="n">
-        <v>5875.71</v>
+        <v>1496.72</v>
       </c>
       <c r="G17" s="2" t="n">
         <v>0</v>
@@ -2632,20 +2932,20 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>PAREDES ORTIZ MARIA INES</t>
+          <t>MANABITA DE REPUESTOS MANARECO C LTDA</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>8791.290000000001</v>
+        <v>0</v>
       </c>
       <c r="E18" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F18" s="2" t="n">
-        <v>2719.84</v>
+        <v>0</v>
       </c>
       <c r="G18" s="2" t="n">
         <v>0</v>
@@ -2659,20 +2959,20 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>RENOVA&amp;DISEÑA S.A.</t>
+          <t>MATERIALES PARA DECORACION DECORCASA CIA. LTDA.</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>253.44</v>
+        <v>0</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>0</v>
+        <v>835.22</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>96.37</v>
+        <v>0</v>
       </c>
       <c r="F19" s="2" t="n">
-        <v>1222.16</v>
+        <v>3124.48</v>
       </c>
       <c r="G19" s="2" t="n">
         <v>0</v>
@@ -2686,11 +2986,11 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>REYES AGUILERA JESSICA ELIZABETH</t>
+          <t>MOREIRA MOREIRA PATRICIO IGNACIO</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>0</v>
+        <v>89.76000000000001</v>
       </c>
       <c r="D20" s="2" t="n">
         <v>0</v>
@@ -2699,7 +2999,7 @@
         <v>0</v>
       </c>
       <c r="F20" s="2" t="n">
-        <v>0</v>
+        <v>5875.71</v>
       </c>
       <c r="G20" s="2" t="n">
         <v>0</v>
@@ -2713,20 +3013,20 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>ROCA REYNA PAUL DAVID</t>
+          <t>PAREDES ORTIZ MARIA INES</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>1391.04</v>
+        <v>0</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>4780.84</v>
+        <v>8791.290000000001</v>
       </c>
       <c r="E21" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F21" s="2" t="n">
-        <v>0</v>
+        <v>2719.84</v>
       </c>
       <c r="G21" s="2" t="n">
         <v>0</v>
@@ -2740,20 +3040,20 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>SUMBA GARCIA MARCOS ANTONIO</t>
+          <t>RENOVA&amp;DISEÑA S.A.</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>0</v>
+        <v>253.44</v>
       </c>
       <c r="D22" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E22" s="2" t="n">
-        <v>0</v>
+        <v>96.37</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>0</v>
+        <v>1222.16</v>
       </c>
       <c r="G22" s="2" t="n">
         <v>0</v>
@@ -2767,7 +3067,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>TUTIVEN PAREDES MARCIA PIEDAD</t>
+          <t>REYES AGUILERA JESSICA ELIZABETH</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
@@ -2794,14 +3094,14 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>VACA CANCHINGRE FATIMA YAQUELINE</t>
+          <t>ROCA REYNA PAUL DAVID</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>0</v>
+        <v>1391.04</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>0</v>
+        <v>4780.84</v>
       </c>
       <c r="E24" s="2" t="n">
         <v>0</v>
@@ -2821,7 +3121,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>ZAMBRANO FERNANDEZ JOSE LUIS</t>
+          <t>SOLORZANO BRAVO TERESA CONCEPCION</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
@@ -2848,39 +3148,174 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
+          <t>SUMBA GARCIA MARCOS ANTONIO</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>MEZA PEÑA CARLOS ROBERTO</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>TUTIVEN PAREDES MARCIA PIEDAD</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>MEZA PEÑA CARLOS ROBERTO</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>VACA CANCHINGRE FATIMA YAQUELINE</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G28" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>MEZA PEÑA CARLOS ROBERTO</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>VERA ARCE MARIA ISABEL</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>MEZA PEÑA CARLOS ROBERTO</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>ZAMBRANO FERNANDEZ JOSE LUIS</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>MEZA PEÑA CARLOS ROBERTO</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
           <t>ZAMBRANO REYNA JOSE ALEJANDRO</t>
         </is>
       </c>
-      <c r="C26" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D26" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E26" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F26" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G26" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="C27" s="4" t="n">
+      <c r="C31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="C32" s="4" t="n">
         <v>3836.67</v>
       </c>
-      <c r="D27" s="4" t="n">
+      <c r="D32" s="4" t="n">
         <v>14896.46</v>
       </c>
-      <c r="E27" s="4" t="n">
+      <c r="E32" s="4" t="n">
         <v>96.37</v>
       </c>
-      <c r="F27" s="4" t="n">
+      <c r="F32" s="4" t="n">
         <v>14994.32</v>
       </c>
-      <c r="G27" s="4" t="n">
+      <c r="G32" s="4" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática 2026-01-29 08:30:10
</commit_message>
<xml_diff>
--- a/data/MEZA PEÑA CARLOS ROBERTO.xlsx
+++ b/data/MEZA PEÑA CARLOS ROBERTO.xlsx
@@ -440,11 +440,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R32"/>
+  <dimension ref="A1:R33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="49" customWidth="1" min="2" max="2"/>
+    <col width="53" customWidth="1" min="2" max="2"/>
     <col width="25" customWidth="1" min="3" max="3"/>
     <col width="24" customWidth="1" min="4" max="4"/>
     <col width="26" customWidth="1" min="5" max="5"/>
@@ -1283,7 +1283,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>FREILE FERRIN FRECIA NOEMI LOURDE</t>
+          <t>FRANQUICIA DISTRIBUIDORA SANTA MARIA FRADISAMA S.A.</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
@@ -1343,7 +1343,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>GONZALEZ CARDENAS ERNESTO PAOLO</t>
+          <t>FREILE FERRIN FRECIA NOEMI LOURDE</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
@@ -1403,7 +1403,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>GRANIMUNDO S.A.</t>
+          <t>GONZALEZ CARDENAS ERNESTO PAOLO</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
@@ -1413,7 +1413,7 @@
         <v>0</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>166.61</v>
+        <v>0</v>
       </c>
       <c r="F16" s="2" t="n">
         <v>0</v>
@@ -1463,7 +1463,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>LINO TUMBACO VICENTE JAVIER</t>
+          <t>GRANIMUNDO S.A.</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
@@ -1473,7 +1473,7 @@
         <v>0</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>0</v>
+        <v>166.61</v>
       </c>
       <c r="F17" s="2" t="n">
         <v>0</v>
@@ -1497,7 +1497,7 @@
         <v>0</v>
       </c>
       <c r="M17" s="2" t="n">
-        <v>1496.72</v>
+        <v>0</v>
       </c>
       <c r="N17" s="2" t="n">
         <v>0</v>
@@ -1523,7 +1523,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>MANABITA DE REPUESTOS MANARECO C LTDA</t>
+          <t>LINO TUMBACO VICENTE JAVIER</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
@@ -1557,7 +1557,7 @@
         <v>0</v>
       </c>
       <c r="M18" s="2" t="n">
-        <v>0</v>
+        <v>1496.72</v>
       </c>
       <c r="N18" s="2" t="n">
         <v>0</v>
@@ -1583,7 +1583,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>MATERIALES PARA DECORACION DECORCASA CIA. LTDA.</t>
+          <t>MANABITA DE REPUESTOS MANARECO C LTDA</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
@@ -1617,7 +1617,7 @@
         <v>0</v>
       </c>
       <c r="M19" s="2" t="n">
-        <v>3124.48</v>
+        <v>0</v>
       </c>
       <c r="N19" s="2" t="n">
         <v>0</v>
@@ -1643,17 +1643,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>MOREIRA MOREIRA PATRICIO IGNACIO</t>
+          <t>MATERIALES PARA DECORACION DECORCASA CIA. LTDA.</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>1166.4</v>
+        <v>0</v>
       </c>
       <c r="D20" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>867.5599999999999</v>
+        <v>0</v>
       </c>
       <c r="F20" s="2" t="n">
         <v>0</v>
@@ -1674,10 +1674,10 @@
         <v>0</v>
       </c>
       <c r="L20" s="2" t="n">
-        <v>2345.61</v>
+        <v>0</v>
       </c>
       <c r="M20" s="2" t="n">
-        <v>1496.14</v>
+        <v>3124.48</v>
       </c>
       <c r="N20" s="2" t="n">
         <v>0</v>
@@ -1703,17 +1703,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>PAREDES ORTIZ MARIA INES</t>
+          <t>MOREIRA MOREIRA PATRICIO IGNACIO</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>0</v>
+        <v>1166.4</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>2719.84</v>
+        <v>0</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>0</v>
+        <v>867.5599999999999</v>
       </c>
       <c r="F21" s="2" t="n">
         <v>0</v>
@@ -1734,10 +1734,10 @@
         <v>0</v>
       </c>
       <c r="L21" s="2" t="n">
-        <v>0</v>
+        <v>2345.61</v>
       </c>
       <c r="M21" s="2" t="n">
-        <v>0</v>
+        <v>1496.14</v>
       </c>
       <c r="N21" s="2" t="n">
         <v>0</v>
@@ -1763,14 +1763,14 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>RENOVA&amp;DISEÑA S.A.</t>
+          <t>PAREDES ORTIZ MARIA INES</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>630.91</v>
+        <v>2719.84</v>
       </c>
       <c r="E22" s="2" t="n">
         <v>0</v>
@@ -1794,7 +1794,7 @@
         <v>0</v>
       </c>
       <c r="L22" s="2" t="n">
-        <v>591.25</v>
+        <v>0</v>
       </c>
       <c r="M22" s="2" t="n">
         <v>0</v>
@@ -1823,14 +1823,14 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>REYES AGUILERA JESSICA ELIZABETH</t>
+          <t>RENOVA&amp;DISEÑA S.A.</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>0</v>
+        <v>630.91</v>
       </c>
       <c r="E23" s="2" t="n">
         <v>0</v>
@@ -1854,7 +1854,7 @@
         <v>0</v>
       </c>
       <c r="L23" s="2" t="n">
-        <v>0</v>
+        <v>591.25</v>
       </c>
       <c r="M23" s="2" t="n">
         <v>0</v>
@@ -1883,7 +1883,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>ROCA REYNA PAUL DAVID</t>
+          <t>REYES AGUILERA JESSICA ELIZABETH</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
@@ -1943,7 +1943,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>SOLORZANO BRAVO TERESA CONCEPCION</t>
+          <t>ROCA REYNA PAUL DAVID</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
@@ -2003,7 +2003,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>SUMBA GARCIA MARCOS ANTONIO</t>
+          <t>SOLORZANO BRAVO TERESA CONCEPCION</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
@@ -2063,7 +2063,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>TUTIVEN PAREDES MARCIA PIEDAD</t>
+          <t>SUMBA GARCIA MARCOS ANTONIO</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
@@ -2123,7 +2123,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>VACA CANCHINGRE FATIMA YAQUELINE</t>
+          <t>TUTIVEN PAREDES MARCIA PIEDAD</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
@@ -2183,7 +2183,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>VERA ARCE MARIA ISABEL</t>
+          <t>VACA CANCHINGRE FATIMA YAQUELINE</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
@@ -2243,7 +2243,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>ZAMBRANO FERNANDEZ JOSE LUIS</t>
+          <t>VERA ARCE MARIA ISABEL</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
@@ -2303,137 +2303,197 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
+          <t>ZAMBRANO FERNANDEZ JOSE LUIS</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R31" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>MEZA PEÑA CARLOS ROBERTO</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
           <t>ZAMBRANO REYNA JOSE ALEJANDRO</t>
         </is>
       </c>
-      <c r="C31" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D31" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E31" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F31" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G31" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H31" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I31" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J31" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K31" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L31" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M31" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N31" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O31" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P31" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q31" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R31" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="C32" s="3" t="inlineStr">
-        <is>
-          <t>1 de 30</t>
-        </is>
-      </c>
-      <c r="D32" s="3" t="inlineStr">
-        <is>
-          <t>2 de 30</t>
-        </is>
-      </c>
-      <c r="E32" s="3" t="inlineStr">
-        <is>
-          <t>2 de 30</t>
-        </is>
-      </c>
-      <c r="F32" s="3" t="inlineStr">
-        <is>
-          <t>0 de 30</t>
-        </is>
-      </c>
-      <c r="G32" s="3" t="inlineStr">
-        <is>
-          <t>0 de 30</t>
-        </is>
-      </c>
-      <c r="H32" s="3" t="inlineStr">
-        <is>
-          <t>1 de 30</t>
-        </is>
-      </c>
-      <c r="I32" s="3" t="inlineStr">
-        <is>
-          <t>1 de 30</t>
-        </is>
-      </c>
-      <c r="J32" s="3" t="inlineStr">
-        <is>
-          <t>0 de 30</t>
-        </is>
-      </c>
-      <c r="K32" s="3" t="inlineStr">
-        <is>
-          <t>0 de 30</t>
-        </is>
-      </c>
-      <c r="L32" s="3" t="inlineStr">
-        <is>
-          <t>2 de 30</t>
-        </is>
-      </c>
-      <c r="M32" s="3" t="inlineStr">
-        <is>
-          <t>3 de 30</t>
-        </is>
-      </c>
-      <c r="N32" s="3" t="inlineStr">
-        <is>
-          <t>0 de 30</t>
-        </is>
-      </c>
-      <c r="O32" s="3" t="inlineStr">
-        <is>
-          <t>0 de 30</t>
-        </is>
-      </c>
-      <c r="P32" s="3" t="inlineStr">
-        <is>
-          <t>0 de 30</t>
-        </is>
-      </c>
-      <c r="Q32" s="3" t="inlineStr">
-        <is>
-          <t>0 de 30</t>
-        </is>
-      </c>
-      <c r="R32" s="3" t="inlineStr">
-        <is>
-          <t>0 de 30</t>
+      <c r="C32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R32" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>1 de 31</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>2 de 31</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>2 de 31</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>0 de 31</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>0 de 31</t>
+        </is>
+      </c>
+      <c r="H33" s="3" t="inlineStr">
+        <is>
+          <t>1 de 31</t>
+        </is>
+      </c>
+      <c r="I33" s="3" t="inlineStr">
+        <is>
+          <t>1 de 31</t>
+        </is>
+      </c>
+      <c r="J33" s="3" t="inlineStr">
+        <is>
+          <t>0 de 31</t>
+        </is>
+      </c>
+      <c r="K33" s="3" t="inlineStr">
+        <is>
+          <t>0 de 31</t>
+        </is>
+      </c>
+      <c r="L33" s="3" t="inlineStr">
+        <is>
+          <t>2 de 31</t>
+        </is>
+      </c>
+      <c r="M33" s="3" t="inlineStr">
+        <is>
+          <t>3 de 31</t>
+        </is>
+      </c>
+      <c r="N33" s="3" t="inlineStr">
+        <is>
+          <t>0 de 31</t>
+        </is>
+      </c>
+      <c r="O33" s="3" t="inlineStr">
+        <is>
+          <t>0 de 31</t>
+        </is>
+      </c>
+      <c r="P33" s="3" t="inlineStr">
+        <is>
+          <t>0 de 31</t>
+        </is>
+      </c>
+      <c r="Q33" s="3" t="inlineStr">
+        <is>
+          <t>0 de 31</t>
+        </is>
+      </c>
+      <c r="R33" s="3" t="inlineStr">
+        <is>
+          <t>0 de 31</t>
         </is>
       </c>
     </row>
@@ -2448,11 +2508,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="49" customWidth="1" min="2" max="2"/>
+    <col width="53" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
@@ -2829,7 +2889,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>FREILE FERRIN FRECIA NOEMI LOURDE</t>
+          <t>FRANQUICIA DISTRIBUIDORA SANTA MARIA FRADISAMA S.A.</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
@@ -2856,7 +2916,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>GONZALEZ CARDENAS ERNESTO PAOLO</t>
+          <t>FREILE FERRIN FRECIA NOEMI LOURDE</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
@@ -2883,11 +2943,11 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>GRANIMUNDO S.A.</t>
+          <t>GONZALEZ CARDENAS ERNESTO PAOLO</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>1382.33</v>
+        <v>0</v>
       </c>
       <c r="D16" s="2" t="n">
         <v>0</v>
@@ -2896,7 +2956,7 @@
         <v>0</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>166.61</v>
+        <v>0</v>
       </c>
       <c r="G16" s="2" t="n">
         <v>0</v>
@@ -2910,11 +2970,11 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>LINO TUMBACO VICENTE JAVIER</t>
+          <t>GRANIMUNDO S.A.</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>0</v>
+        <v>1382.33</v>
       </c>
       <c r="D17" s="2" t="n">
         <v>0</v>
@@ -2923,7 +2983,7 @@
         <v>0</v>
       </c>
       <c r="F17" s="2" t="n">
-        <v>1496.72</v>
+        <v>166.61</v>
       </c>
       <c r="G17" s="2" t="n">
         <v>0</v>
@@ -2937,7 +2997,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>MANABITA DE REPUESTOS MANARECO C LTDA</t>
+          <t>LINO TUMBACO VICENTE JAVIER</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
@@ -2950,7 +3010,7 @@
         <v>0</v>
       </c>
       <c r="F18" s="2" t="n">
-        <v>0</v>
+        <v>1496.72</v>
       </c>
       <c r="G18" s="2" t="n">
         <v>0</v>
@@ -2964,20 +3024,20 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>MATERIALES PARA DECORACION DECORCASA CIA. LTDA.</t>
+          <t>MANABITA DE REPUESTOS MANARECO C LTDA</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>835.22</v>
+        <v>0</v>
       </c>
       <c r="E19" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F19" s="2" t="n">
-        <v>3124.48</v>
+        <v>0</v>
       </c>
       <c r="G19" s="2" t="n">
         <v>0</v>
@@ -2991,20 +3051,20 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>MOREIRA MOREIRA PATRICIO IGNACIO</t>
+          <t>MATERIALES PARA DECORACION DECORCASA CIA. LTDA.</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>89.76000000000001</v>
+        <v>0</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>0</v>
+        <v>835.22</v>
       </c>
       <c r="E20" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F20" s="2" t="n">
-        <v>5875.71</v>
+        <v>3124.48</v>
       </c>
       <c r="G20" s="2" t="n">
         <v>0</v>
@@ -3018,20 +3078,20 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>PAREDES ORTIZ MARIA INES</t>
+          <t>MOREIRA MOREIRA PATRICIO IGNACIO</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>0</v>
+        <v>89.76000000000001</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>8791.290000000001</v>
+        <v>0</v>
       </c>
       <c r="E21" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F21" s="2" t="n">
-        <v>2719.84</v>
+        <v>5875.71</v>
       </c>
       <c r="G21" s="2" t="n">
         <v>0</v>
@@ -3045,20 +3105,20 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>RENOVA&amp;DISEÑA S.A.</t>
+          <t>PAREDES ORTIZ MARIA INES</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>253.44</v>
+        <v>0</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>0</v>
+        <v>8791.290000000001</v>
       </c>
       <c r="E22" s="2" t="n">
-        <v>96.37</v>
+        <v>0</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>1222.16</v>
+        <v>2719.84</v>
       </c>
       <c r="G22" s="2" t="n">
         <v>0</v>
@@ -3072,20 +3132,20 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>REYES AGUILERA JESSICA ELIZABETH</t>
+          <t>RENOVA&amp;DISEÑA S.A.</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>0</v>
+        <v>253.44</v>
       </c>
       <c r="D23" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>0</v>
+        <v>96.37</v>
       </c>
       <c r="F23" s="2" t="n">
-        <v>0</v>
+        <v>1222.16</v>
       </c>
       <c r="G23" s="2" t="n">
         <v>0</v>
@@ -3099,14 +3159,14 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>ROCA REYNA PAUL DAVID</t>
+          <t>REYES AGUILERA JESSICA ELIZABETH</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>1391.04</v>
+        <v>0</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>4780.84</v>
+        <v>0</v>
       </c>
       <c r="E24" s="2" t="n">
         <v>0</v>
@@ -3126,14 +3186,14 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>SOLORZANO BRAVO TERESA CONCEPCION</t>
+          <t>ROCA REYNA PAUL DAVID</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>0</v>
+        <v>1391.04</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>0</v>
+        <v>4780.84</v>
       </c>
       <c r="E25" s="2" t="n">
         <v>0</v>
@@ -3153,7 +3213,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>SUMBA GARCIA MARCOS ANTONIO</t>
+          <t>SOLORZANO BRAVO TERESA CONCEPCION</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
@@ -3180,7 +3240,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>TUTIVEN PAREDES MARCIA PIEDAD</t>
+          <t>SUMBA GARCIA MARCOS ANTONIO</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
@@ -3207,7 +3267,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>VACA CANCHINGRE FATIMA YAQUELINE</t>
+          <t>TUTIVEN PAREDES MARCIA PIEDAD</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
@@ -3234,7 +3294,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>VERA ARCE MARIA ISABEL</t>
+          <t>VACA CANCHINGRE FATIMA YAQUELINE</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
@@ -3261,7 +3321,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>ZAMBRANO FERNANDEZ JOSE LUIS</t>
+          <t>VERA ARCE MARIA ISABEL</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
@@ -3288,39 +3348,66 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
+          <t>ZAMBRANO FERNANDEZ JOSE LUIS</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>MEZA PEÑA CARLOS ROBERTO</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
           <t>ZAMBRANO REYNA JOSE ALEJANDRO</t>
         </is>
       </c>
-      <c r="C31" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D31" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E31" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F31" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G31" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="C32" s="4" t="n">
+      <c r="C32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G32" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="C33" s="4" t="n">
         <v>3836.67</v>
       </c>
-      <c r="D32" s="4" t="n">
+      <c r="D33" s="4" t="n">
         <v>14896.46</v>
       </c>
-      <c r="E32" s="4" t="n">
+      <c r="E33" s="4" t="n">
         <v>96.37</v>
       </c>
-      <c r="F32" s="4" t="n">
+      <c r="F33" s="4" t="n">
         <v>14994.32</v>
       </c>
-      <c r="G32" s="4" t="n">
+      <c r="G33" s="4" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática 2026-02-23 17:30:24
</commit_message>
<xml_diff>
--- a/data/MEZA PEÑA CARLOS ROBERTO.xlsx
+++ b/data/MEZA PEÑA CARLOS ROBERTO.xlsx
@@ -1842,7 +1842,7 @@
         <v>0</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>0</v>
+        <v>782.1</v>
       </c>
       <c r="I23" s="2" t="n">
         <v>0</v>
@@ -1857,7 +1857,7 @@
         <v>0</v>
       </c>
       <c r="M23" s="2" t="n">
-        <v>1388.02</v>
+        <v>5378.75</v>
       </c>
       <c r="N23" s="2" t="n">
         <v>0</v>
@@ -2443,7 +2443,7 @@
       </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
-          <t>1 de 31</t>
+          <t>2 de 31</t>
         </is>
       </c>
       <c r="I33" s="3" t="inlineStr">
@@ -3145,7 +3145,7 @@
         <v>1442.48</v>
       </c>
       <c r="F23" s="2" t="n">
-        <v>1388.02</v>
+        <v>6160.85</v>
       </c>
       <c r="G23" s="2" t="n">
         <v>0</v>
@@ -3405,7 +3405,7 @@
         <v>17721.81</v>
       </c>
       <c r="F33" s="4" t="n">
-        <v>7962.35</v>
+        <v>12735.18</v>
       </c>
       <c r="G33" s="4" t="n">
         <v>0</v>
@@ -3480,10 +3480,10 @@
         <v>0</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>5759.92</v>
+        <v>6542.02</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>-5759.92</v>
+        <v>-6542.02</v>
       </c>
       <c r="F2" s="5" t="n">
         <v>0</v>
@@ -3528,13 +3528,13 @@
         <v>10350</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>2202.43</v>
+        <v>6193.16</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>8147.57</v>
+        <v>4156.84</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>0.2127951690821256</v>
+        <v>0.5983729468599034</v>
       </c>
     </row>
     <row r="5">
@@ -3547,13 +3547,13 @@
         <v>10465</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>7962.35</v>
+        <v>12735.18</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>2502.65</v>
+        <v>-2270.18</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.760855231724797</v>
+        <v>1.216930721452461</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-02-27 08:30:20
</commit_message>
<xml_diff>
--- a/data/MEZA PEÑA CARLOS ROBERTO.xlsx
+++ b/data/MEZA PEÑA CARLOS ROBERTO.xlsx
@@ -1470,7 +1470,7 @@
         <v>0</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>0</v>
+        <v>610.5599999999999</v>
       </c>
       <c r="E17" s="2" t="n">
         <v>0</v>
@@ -1857,7 +1857,7 @@
         <v>0</v>
       </c>
       <c r="M23" s="2" t="n">
-        <v>5378.75</v>
+        <v>5397.84</v>
       </c>
       <c r="N23" s="2" t="n">
         <v>0</v>
@@ -2423,7 +2423,7 @@
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>1 de 31</t>
+          <t>2 de 31</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
@@ -2983,7 +2983,7 @@
         <v>2198.58</v>
       </c>
       <c r="F17" s="2" t="n">
-        <v>0</v>
+        <v>610.5599999999999</v>
       </c>
       <c r="G17" s="2" t="n">
         <v>0</v>
@@ -3145,7 +3145,7 @@
         <v>1442.48</v>
       </c>
       <c r="F23" s="2" t="n">
-        <v>6160.85</v>
+        <v>6179.94</v>
       </c>
       <c r="G23" s="2" t="n">
         <v>0</v>
@@ -3405,7 +3405,7 @@
         <v>17721.81</v>
       </c>
       <c r="F33" s="4" t="n">
-        <v>12715.79</v>
+        <v>13345.44</v>
       </c>
       <c r="G33" s="4" t="n">
         <v>0</v>
@@ -3480,10 +3480,10 @@
         <v>0</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>6522.63</v>
+        <v>7133.19</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>-6522.63</v>
+        <v>-7133.19</v>
       </c>
       <c r="F2" s="5" t="n">
         <v>0</v>
@@ -3528,13 +3528,13 @@
         <v>10350</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>6193.16</v>
+        <v>6217.65</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>4156.84</v>
+        <v>4132.35</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>0.5983729468599034</v>
+        <v>0.6007391304347826</v>
       </c>
     </row>
     <row r="5">
@@ -3547,13 +3547,13 @@
         <v>10465</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>12715.79</v>
+        <v>13350.84</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>-2250.79</v>
+        <v>-2885.839999999999</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>1.215077878643096</v>
+        <v>1.275761108456761</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-03-24 12:30:24
</commit_message>
<xml_diff>
--- a/data/MEZA PEÑA CARLOS ROBERTO.xlsx
+++ b/data/MEZA PEÑA CARLOS ROBERTO.xlsx
@@ -1854,7 +1854,7 @@
         <v>0</v>
       </c>
       <c r="L23" s="2" t="n">
-        <v>0</v>
+        <v>556.8099999999999</v>
       </c>
       <c r="M23" s="2" t="n">
         <v>144.56</v>
@@ -2463,7 +2463,7 @@
       </c>
       <c r="L33" s="3" t="inlineStr">
         <is>
-          <t>0 de 31</t>
+          <t>1 de 31</t>
         </is>
       </c>
       <c r="M33" s="3" t="inlineStr">
@@ -3145,7 +3145,7 @@
         <v>6179.94</v>
       </c>
       <c r="F23" s="2" t="n">
-        <v>425.36</v>
+        <v>982.17</v>
       </c>
       <c r="G23" s="2" t="n">
         <v>0</v>
@@ -3405,7 +3405,7 @@
         <v>13604.64</v>
       </c>
       <c r="F33" s="4" t="n">
-        <v>425.36</v>
+        <v>982.17</v>
       </c>
       <c r="G33" s="4" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Actualización automática 2026-04-07 17:30:19
</commit_message>
<xml_diff>
--- a/data/MEZA PEÑA CARLOS ROBERTO.xlsx
+++ b/data/MEZA PEÑA CARLOS ROBERTO.xlsx
@@ -1677,7 +1677,7 @@
         <v>0</v>
       </c>
       <c r="M20" s="2" t="n">
-        <v>0</v>
+        <v>51.97</v>
       </c>
       <c r="N20" s="2" t="n">
         <v>0</v>
@@ -2468,7 +2468,7 @@
       </c>
       <c r="M33" s="3" t="inlineStr">
         <is>
-          <t>0 de 31</t>
+          <t>1 de 31</t>
         </is>
       </c>
       <c r="N33" s="3" t="inlineStr">
@@ -3064,7 +3064,7 @@
         <v>5608.65</v>
       </c>
       <c r="F20" s="2" t="n">
-        <v>0</v>
+        <v>51.97</v>
       </c>
       <c r="G20" s="2" t="n">
         <v>0</v>
@@ -3405,7 +3405,7 @@
         <v>15442.93</v>
       </c>
       <c r="F33" s="4" t="n">
-        <v>-51.54</v>
+        <v>0.4299999999999997</v>
       </c>
       <c r="G33" s="4" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Actualización automática 2026-04-13 11:30:21
</commit_message>
<xml_diff>
--- a/data/MEZA PEÑA CARLOS ROBERTO.xlsx
+++ b/data/MEZA PEÑA CARLOS ROBERTO.xlsx
@@ -1677,7 +1677,7 @@
         <v>0</v>
       </c>
       <c r="M20" s="2" t="n">
-        <v>51.97</v>
+        <v>120.83</v>
       </c>
       <c r="N20" s="2" t="n">
         <v>0</v>
@@ -1986,7 +1986,7 @@
         <v>0</v>
       </c>
       <c r="P25" s="2" t="n">
-        <v>0</v>
+        <v>174.6</v>
       </c>
       <c r="Q25" s="2" t="n">
         <v>0</v>
@@ -2483,7 +2483,7 @@
       </c>
       <c r="P33" s="3" t="inlineStr">
         <is>
-          <t>0 de 31</t>
+          <t>1 de 31</t>
         </is>
       </c>
       <c r="Q33" s="3" t="inlineStr">
@@ -3064,7 +3064,7 @@
         <v>5608.65</v>
       </c>
       <c r="F20" s="2" t="n">
-        <v>51.97</v>
+        <v>120.83</v>
       </c>
       <c r="G20" s="2" t="n">
         <v>0</v>
@@ -3199,7 +3199,7 @@
         <v>3034.32</v>
       </c>
       <c r="F25" s="2" t="n">
-        <v>0</v>
+        <v>174.6</v>
       </c>
       <c r="G25" s="2" t="n">
         <v>0</v>
@@ -3405,7 +3405,7 @@
         <v>15442.93</v>
       </c>
       <c r="F33" s="4" t="n">
-        <v>625.98</v>
+        <v>869.4399999999999</v>
       </c>
       <c r="G33" s="4" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Actualización automática 2026-04-21 12:30:23
</commit_message>
<xml_diff>
--- a/data/MEZA PEÑA CARLOS ROBERTO.xlsx
+++ b/data/MEZA PEÑA CARLOS ROBERTO.xlsx
@@ -1950,7 +1950,7 @@
         <v>0</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>0</v>
+        <v>472.09</v>
       </c>
       <c r="E25" s="2" t="n">
         <v>0</v>
@@ -2423,7 +2423,7 @@
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>0 de 31</t>
+          <t>1 de 31</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
@@ -3199,7 +3199,7 @@
         <v>3034.32</v>
       </c>
       <c r="F25" s="2" t="n">
-        <v>1088.88</v>
+        <v>1560.97</v>
       </c>
       <c r="G25" s="2" t="n">
         <v>0</v>
@@ -3405,7 +3405,7 @@
         <v>15442.93</v>
       </c>
       <c r="F33" s="4" t="n">
-        <v>2136.23</v>
+        <v>2608.32</v>
       </c>
       <c r="G33" s="4" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Actualización automática 2026-05-04 15:30:19
</commit_message>
<xml_diff>
--- a/data/MEZA PEÑA CARLOS ROBERTO.xlsx
+++ b/data/MEZA PEÑA CARLOS ROBERTO.xlsx
@@ -1854,7 +1854,7 @@
         <v>0</v>
       </c>
       <c r="L23" s="2" t="n">
-        <v>0</v>
+        <v>170.48</v>
       </c>
       <c r="M23" s="2" t="n">
         <v>0</v>
@@ -2463,7 +2463,7 @@
       </c>
       <c r="L33" s="3" t="inlineStr">
         <is>
-          <t>0 de 31</t>
+          <t>1 de 31</t>
         </is>
       </c>
       <c r="M33" s="3" t="inlineStr">
@@ -2516,7 +2516,7 @@
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -3145,7 +3145,7 @@
         <v>2195.57</v>
       </c>
       <c r="F23" s="2" t="n">
-        <v>0</v>
+        <v>170.48</v>
       </c>
       <c r="G23" s="2" t="n">
         <v>0</v>
@@ -3405,7 +3405,7 @@
         <v>4885.37</v>
       </c>
       <c r="F33" s="4" t="n">
-        <v>0</v>
+        <v>170.48</v>
       </c>
       <c r="G33" s="4" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Actualización automática 2026-05-27 09:30:28
</commit_message>
<xml_diff>
--- a/data/MEZA PEÑA CARLOS ROBERTO.xlsx
+++ b/data/MEZA PEÑA CARLOS ROBERTO.xlsx
@@ -1587,10 +1587,10 @@
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>0</v>
+        <v>1497.6</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>0</v>
+        <v>1603.3</v>
       </c>
       <c r="E19" s="2" t="n">
         <v>0</v>
@@ -1614,7 +1614,7 @@
         <v>0</v>
       </c>
       <c r="L19" s="2" t="n">
-        <v>0</v>
+        <v>2377.58</v>
       </c>
       <c r="M19" s="2" t="n">
         <v>0</v>
@@ -2298,52 +2298,52 @@
     <row r="31">
       <c r="C31" s="3" t="inlineStr">
         <is>
+          <t>1 de 29</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>1 de 29</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
           <t>0 de 29</t>
         </is>
       </c>
-      <c r="D31" s="3" t="inlineStr">
+      <c r="F31" s="3" t="inlineStr">
         <is>
           <t>0 de 29</t>
         </is>
       </c>
-      <c r="E31" s="3" t="inlineStr">
+      <c r="G31" s="3" t="inlineStr">
         <is>
           <t>0 de 29</t>
         </is>
       </c>
-      <c r="F31" s="3" t="inlineStr">
+      <c r="H31" s="3" t="inlineStr">
         <is>
           <t>0 de 29</t>
         </is>
       </c>
-      <c r="G31" s="3" t="inlineStr">
+      <c r="I31" s="3" t="inlineStr">
         <is>
           <t>0 de 29</t>
         </is>
       </c>
-      <c r="H31" s="3" t="inlineStr">
+      <c r="J31" s="3" t="inlineStr">
         <is>
           <t>0 de 29</t>
         </is>
       </c>
-      <c r="I31" s="3" t="inlineStr">
+      <c r="K31" s="3" t="inlineStr">
         <is>
           <t>0 de 29</t>
         </is>
       </c>
-      <c r="J31" s="3" t="inlineStr">
-        <is>
-          <t>0 de 29</t>
-        </is>
-      </c>
-      <c r="K31" s="3" t="inlineStr">
-        <is>
-          <t>0 de 29</t>
-        </is>
-      </c>
       <c r="L31" s="3" t="inlineStr">
         <is>
-          <t>1 de 29</t>
+          <t>2 de 29</t>
         </is>
       </c>
       <c r="M31" s="3" t="inlineStr">
@@ -3025,7 +3025,7 @@
         <v>0</v>
       </c>
       <c r="F23" s="2" t="n">
-        <v>0</v>
+        <v>5478.48</v>
       </c>
       <c r="G23" s="2" t="n">
         <v>0</v>
@@ -3393,7 +3393,7 @@
         <v>4885.37</v>
       </c>
       <c r="F37" s="4" t="n">
-        <v>1293.56</v>
+        <v>6772.039999999999</v>
       </c>
       <c r="G37" s="4" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Actualización automática 2026-05-27 12:30:23
</commit_message>
<xml_diff>
--- a/data/MEZA PEÑA CARLOS ROBERTO.xlsx
+++ b/data/MEZA PEÑA CARLOS ROBERTO.xlsx
@@ -1710,7 +1710,7 @@
         <v>0</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>0</v>
+        <v>2203.08</v>
       </c>
       <c r="E21" s="2" t="n">
         <v>0</v>
@@ -2303,7 +2303,7 @@
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>1 de 29</t>
+          <t>2 de 29</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
@@ -3079,7 +3079,7 @@
         <v>2195.57</v>
       </c>
       <c r="F25" s="2" t="n">
-        <v>1293.56</v>
+        <v>3496.64</v>
       </c>
       <c r="G25" s="2" t="n">
         <v>0</v>
@@ -3393,7 +3393,7 @@
         <v>4885.37</v>
       </c>
       <c r="F37" s="4" t="n">
-        <v>12853.5</v>
+        <v>15056.58</v>
       </c>
       <c r="G37" s="4" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Actualización automática 2026-06-04 17:30:22
</commit_message>
<xml_diff>
--- a/data/MEZA PEÑA CARLOS ROBERTO.xlsx
+++ b/data/MEZA PEÑA CARLOS ROBERTO.xlsx
@@ -1440,7 +1440,7 @@
         <v>0</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>0</v>
+        <v>2971.8</v>
       </c>
       <c r="O16" s="2" t="n">
         <v>0</v>
@@ -1830,7 +1830,7 @@
         <v>0</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>0</v>
+        <v>89.17</v>
       </c>
       <c r="E23" s="2" t="n">
         <v>0</v>
@@ -1854,13 +1854,13 @@
         <v>0</v>
       </c>
       <c r="L23" s="2" t="n">
-        <v>0</v>
+        <v>1103</v>
       </c>
       <c r="M23" s="2" t="n">
         <v>0</v>
       </c>
       <c r="N23" s="2" t="n">
-        <v>0</v>
+        <v>1598.51</v>
       </c>
       <c r="O23" s="2" t="n">
         <v>0</v>
@@ -2303,57 +2303,57 @@
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
+          <t>1 de 29</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
           <t>0 de 29</t>
         </is>
       </c>
-      <c r="E31" s="3" t="inlineStr">
+      <c r="F31" s="3" t="inlineStr">
         <is>
           <t>0 de 29</t>
         </is>
       </c>
-      <c r="F31" s="3" t="inlineStr">
+      <c r="G31" s="3" t="inlineStr">
         <is>
           <t>0 de 29</t>
         </is>
       </c>
-      <c r="G31" s="3" t="inlineStr">
+      <c r="H31" s="3" t="inlineStr">
         <is>
           <t>0 de 29</t>
         </is>
       </c>
-      <c r="H31" s="3" t="inlineStr">
+      <c r="I31" s="3" t="inlineStr">
         <is>
           <t>0 de 29</t>
         </is>
       </c>
-      <c r="I31" s="3" t="inlineStr">
+      <c r="J31" s="3" t="inlineStr">
         <is>
           <t>0 de 29</t>
         </is>
       </c>
-      <c r="J31" s="3" t="inlineStr">
+      <c r="K31" s="3" t="inlineStr">
         <is>
           <t>0 de 29</t>
         </is>
       </c>
-      <c r="K31" s="3" t="inlineStr">
+      <c r="L31" s="3" t="inlineStr">
+        <is>
+          <t>1 de 29</t>
+        </is>
+      </c>
+      <c r="M31" s="3" t="inlineStr">
         <is>
           <t>0 de 29</t>
         </is>
       </c>
-      <c r="L31" s="3" t="inlineStr">
-        <is>
-          <t>0 de 29</t>
-        </is>
-      </c>
-      <c r="M31" s="3" t="inlineStr">
-        <is>
-          <t>0 de 29</t>
-        </is>
-      </c>
       <c r="N31" s="3" t="inlineStr">
         <is>
-          <t>0 de 29</t>
+          <t>2 de 29</t>
         </is>
       </c>
       <c r="O31" s="3" t="inlineStr">
@@ -2396,7 +2396,7 @@
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -2944,7 +2944,7 @@
         <v>249.03</v>
       </c>
       <c r="F20" s="2" t="n">
-        <v>0</v>
+        <v>2971.8</v>
       </c>
       <c r="G20" s="2" t="n">
         <v>0</v>
@@ -3133,7 +3133,7 @@
         <v>0</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>0</v>
+        <v>2790.68</v>
       </c>
       <c r="G27" s="2" t="n">
         <v>0</v>
@@ -3393,7 +3393,7 @@
         <v>33105.81</v>
       </c>
       <c r="F37" s="4" t="n">
-        <v>0</v>
+        <v>5762.48</v>
       </c>
       <c r="G37" s="4" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Actualización automática 2026-06-09 08:30:19
</commit_message>
<xml_diff>
--- a/data/MEZA PEÑA CARLOS ROBERTO.xlsx
+++ b/data/MEZA PEÑA CARLOS ROBERTO.xlsx
@@ -1431,7 +1431,7 @@
         <v>0</v>
       </c>
       <c r="K16" s="2" t="n">
-        <v>0</v>
+        <v>-18.86</v>
       </c>
       <c r="L16" s="2" t="n">
         <v>0</v>
@@ -2944,7 +2944,7 @@
         <v>249.03</v>
       </c>
       <c r="F20" s="2" t="n">
-        <v>2971.8</v>
+        <v>2952.94</v>
       </c>
       <c r="G20" s="2" t="n">
         <v>0</v>
@@ -3393,7 +3393,7 @@
         <v>33105.81</v>
       </c>
       <c r="F37" s="4" t="n">
-        <v>5762.48</v>
+        <v>5743.62</v>
       </c>
       <c r="G37" s="4" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Actualización automática 2026-06-10 10:30:16
</commit_message>
<xml_diff>
--- a/data/MEZA PEÑA CARLOS ROBERTO.xlsx
+++ b/data/MEZA PEÑA CARLOS ROBERTO.xlsx
@@ -1737,7 +1737,7 @@
         <v>0</v>
       </c>
       <c r="M21" s="2" t="n">
-        <v>0</v>
+        <v>31.84</v>
       </c>
       <c r="N21" s="2" t="n">
         <v>0</v>
@@ -2348,7 +2348,7 @@
       </c>
       <c r="M31" s="3" t="inlineStr">
         <is>
-          <t>0 de 29</t>
+          <t>1 de 29</t>
         </is>
       </c>
       <c r="N31" s="3" t="inlineStr">
@@ -3079,7 +3079,7 @@
         <v>17031.68</v>
       </c>
       <c r="F25" s="2" t="n">
-        <v>0</v>
+        <v>31.84</v>
       </c>
       <c r="G25" s="2" t="n">
         <v>0</v>
@@ -3393,7 +3393,7 @@
         <v>33105.81</v>
       </c>
       <c r="F37" s="4" t="n">
-        <v>5743.62</v>
+        <v>5775.46</v>
       </c>
       <c r="G37" s="4" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Actualización automática 2026-06-19 16:30:20
</commit_message>
<xml_diff>
--- a/data/MEZA PEÑA CARLOS ROBERTO.xlsx
+++ b/data/MEZA PEÑA CARLOS ROBERTO.xlsx
@@ -1557,7 +1557,7 @@
         <v>0</v>
       </c>
       <c r="M18" s="2" t="n">
-        <v>0</v>
+        <v>27.39</v>
       </c>
       <c r="N18" s="2" t="n">
         <v>0</v>
@@ -1737,7 +1737,7 @@
         <v>0</v>
       </c>
       <c r="M21" s="2" t="n">
-        <v>31.84</v>
+        <v>38.16</v>
       </c>
       <c r="N21" s="2" t="n">
         <v>0</v>
@@ -2348,7 +2348,7 @@
       </c>
       <c r="M31" s="3" t="inlineStr">
         <is>
-          <t>2 de 29</t>
+          <t>3 de 29</t>
         </is>
       </c>
       <c r="N31" s="3" t="inlineStr">
@@ -2998,7 +2998,7 @@
         <v>0</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>0</v>
+        <v>27.39</v>
       </c>
       <c r="G22" s="2" t="n">
         <v>0</v>
@@ -3079,7 +3079,7 @@
         <v>17031.68</v>
       </c>
       <c r="F25" s="2" t="n">
-        <v>37.24</v>
+        <v>43.56</v>
       </c>
       <c r="G25" s="2" t="n">
         <v>0</v>
@@ -3393,7 +3393,7 @@
         <v>33105.81</v>
       </c>
       <c r="F37" s="4" t="n">
-        <v>14532.27</v>
+        <v>14565.98</v>
       </c>
       <c r="G37" s="4" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Actualización automática 2026-07-03 10:30:15
</commit_message>
<xml_diff>
--- a/data/MEZA PEÑA CARLOS ROBERTO.xlsx
+++ b/data/MEZA PEÑA CARLOS ROBERTO.xlsx
@@ -1557,7 +1557,7 @@
         <v>0</v>
       </c>
       <c r="M18" s="2" t="n">
-        <v>0</v>
+        <v>601.23</v>
       </c>
       <c r="N18" s="2" t="n">
         <v>0</v>
@@ -2348,7 +2348,7 @@
       </c>
       <c r="M31" s="3" t="inlineStr">
         <is>
-          <t>0 de 29</t>
+          <t>1 de 29</t>
         </is>
       </c>
       <c r="N31" s="3" t="inlineStr">
@@ -2396,7 +2396,7 @@
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -2863,7 +2863,7 @@
         <v>27.39</v>
       </c>
       <c r="F17" s="2" t="n">
-        <v>0</v>
+        <v>601.23</v>
       </c>
       <c r="G17" s="2" t="n">
         <v>0</v>
@@ -3231,7 +3231,7 @@
         <v>21103.45</v>
       </c>
       <c r="F31" s="4" t="n">
-        <v>0</v>
+        <v>601.23</v>
       </c>
       <c r="G31" s="4" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Actualización automática 2026-07-24 12:30:19
</commit_message>
<xml_diff>
--- a/data/MEZA PEÑA CARLOS ROBERTO.xlsx
+++ b/data/MEZA PEÑA CARLOS ROBERTO.xlsx
@@ -1647,10 +1647,10 @@
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>0</v>
+        <v>1159.83</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>0</v>
+        <v>6479.42</v>
       </c>
       <c r="E20" s="2" t="n">
         <v>0</v>
@@ -1674,7 +1674,7 @@
         <v>0</v>
       </c>
       <c r="L20" s="2" t="n">
-        <v>0</v>
+        <v>1238.42</v>
       </c>
       <c r="M20" s="2" t="n">
         <v>0</v>
@@ -1854,7 +1854,7 @@
         <v>0</v>
       </c>
       <c r="L23" s="2" t="n">
-        <v>0</v>
+        <v>146.97</v>
       </c>
       <c r="M23" s="2" t="n">
         <v>72.63</v>
@@ -2298,52 +2298,52 @@
     <row r="31">
       <c r="C31" s="3" t="inlineStr">
         <is>
+          <t>1 de 29</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>1 de 29</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
           <t>0 de 29</t>
         </is>
       </c>
-      <c r="D31" s="3" t="inlineStr">
+      <c r="F31" s="3" t="inlineStr">
         <is>
           <t>0 de 29</t>
         </is>
       </c>
-      <c r="E31" s="3" t="inlineStr">
+      <c r="G31" s="3" t="inlineStr">
         <is>
           <t>0 de 29</t>
         </is>
       </c>
-      <c r="F31" s="3" t="inlineStr">
+      <c r="H31" s="3" t="inlineStr">
         <is>
           <t>0 de 29</t>
         </is>
       </c>
-      <c r="G31" s="3" t="inlineStr">
+      <c r="I31" s="3" t="inlineStr">
         <is>
           <t>0 de 29</t>
         </is>
       </c>
-      <c r="H31" s="3" t="inlineStr">
+      <c r="J31" s="3" t="inlineStr">
         <is>
           <t>0 de 29</t>
         </is>
       </c>
-      <c r="I31" s="3" t="inlineStr">
+      <c r="K31" s="3" t="inlineStr">
         <is>
           <t>0 de 29</t>
         </is>
       </c>
-      <c r="J31" s="3" t="inlineStr">
-        <is>
-          <t>0 de 29</t>
-        </is>
-      </c>
-      <c r="K31" s="3" t="inlineStr">
-        <is>
-          <t>0 de 29</t>
-        </is>
-      </c>
       <c r="L31" s="3" t="inlineStr">
         <is>
-          <t>1 de 29</t>
+          <t>3 de 29</t>
         </is>
       </c>
       <c r="M31" s="3" t="inlineStr">
@@ -2396,7 +2396,7 @@
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -2917,7 +2917,7 @@
         <v>6537.47</v>
       </c>
       <c r="F19" s="2" t="n">
-        <v>0</v>
+        <v>8877.67</v>
       </c>
       <c r="G19" s="2" t="n">
         <v>0</v>
@@ -2998,7 +2998,7 @@
         <v>2936.8</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>72.63</v>
+        <v>219.6</v>
       </c>
       <c r="G22" s="2" t="n">
         <v>0</v>
@@ -3231,7 +3231,7 @@
         <v>21103.45</v>
       </c>
       <c r="F31" s="4" t="n">
-        <v>1321.37</v>
+        <v>10346.01</v>
       </c>
       <c r="G31" s="4" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Actualización automática 2026-09-09 14:30:17
</commit_message>
<xml_diff>
--- a/data/MEZA PEÑA CARLOS ROBERTO.xlsx
+++ b/data/MEZA PEÑA CARLOS ROBERTO.xlsx
@@ -1734,7 +1734,7 @@
         <v>0</v>
       </c>
       <c r="L21" s="2" t="n">
-        <v>0</v>
+        <v>457.23</v>
       </c>
       <c r="M21" s="2" t="n">
         <v>0</v>
@@ -2343,7 +2343,7 @@
       </c>
       <c r="L31" s="3" t="inlineStr">
         <is>
-          <t>1 de 29</t>
+          <t>2 de 29</t>
         </is>
       </c>
       <c r="M31" s="3" t="inlineStr">
@@ -2890,7 +2890,7 @@
         <v>888.4</v>
       </c>
       <c r="F18" s="2" t="n">
-        <v>0</v>
+        <v>457.23</v>
       </c>
       <c r="G18" s="2" t="n">
         <v>0</v>
@@ -3177,7 +3177,7 @@
         <v>30461.36</v>
       </c>
       <c r="F29" s="4" t="n">
-        <v>253.96</v>
+        <v>711.1900000000001</v>
       </c>
       <c r="G29" s="4" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Actualización automática 2026-09-10 11:30:18
</commit_message>
<xml_diff>
--- a/data/MEZA PEÑA CARLOS ROBERTO.xlsx
+++ b/data/MEZA PEÑA CARLOS ROBERTO.xlsx
@@ -1557,7 +1557,7 @@
         <v>253.96</v>
       </c>
       <c r="M18" s="2" t="n">
-        <v>0</v>
+        <v>313.63</v>
       </c>
       <c r="N18" s="2" t="n">
         <v>0</v>
@@ -2348,7 +2348,7 @@
       </c>
       <c r="M31" s="3" t="inlineStr">
         <is>
-          <t>0 de 29</t>
+          <t>1 de 29</t>
         </is>
       </c>
       <c r="N31" s="3" t="inlineStr">
@@ -2836,7 +2836,7 @@
         <v>6420.1</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>253.96</v>
+        <v>567.59</v>
       </c>
       <c r="G16" s="2" t="n">
         <v>0</v>
@@ -3204,7 +3204,7 @@
         <v>40471.33</v>
       </c>
       <c r="F30" s="4" t="n">
-        <v>607.1</v>
+        <v>920.73</v>
       </c>
       <c r="G30" s="4" t="n">
         <v>0</v>

</xml_diff>